<commit_message>
Se ejecuta salida de estados en el bloque de datos
</commit_message>
<xml_diff>
--- a/output_SIDCAR/seguimiento_sae_sidcar_grupo_A.xlsx
+++ b/output_SIDCAR/seguimiento_sae_sidcar_grupo_A.xlsx
@@ -21,16 +21,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -41,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -49,21 +46,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -434,182 +422,182 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>expediente</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>nombre_persona</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>funcionario_sae</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>fuentes_presentes</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>en_sae</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>en_preradicados</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>en_radicados</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>etapa_sae</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>actividad_sae</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>ultimo_documento_tipo_sae</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>ultimo_documento_descripcion_sae</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>fecha_ultimo_documento_sae</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>numero_ultimo_documento_sae</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>firmado_por_sae</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>tiene_preradicado</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>numero_preradicado</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>tipo_documento_preradicado</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>estado_preradicado</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>fecha_preradicado</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>asunto_preradicado</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>revisor_pre</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>tiene_radicado</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>numero_radicado</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>tipo_documento_radicado</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>estado_radicado</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>fecha_radicado</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>asunto_radicado</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>preradicado_relacionado</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>revisor_rad</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>fecha_inicio_expediente</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>fecha_fin_expediente</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>dias_transcurridos_expediente</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>estado_vencimiento</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>estado_pelota_caliente</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>revisor_asociado</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>responsable_pelota_caliente</t>
         </is>
@@ -665,7 +653,7 @@
           <t>Oficio de citación</t>
         </is>
       </c>
-      <c r="L2" s="2" t="n">
+      <c r="L2" s="1" t="n">
         <v>46094.6985306713</v>
       </c>
       <c r="M2" t="inlineStr">
@@ -697,7 +685,7 @@
       <c r="AA2" t="inlineStr"/>
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
-      <c r="AD2" s="2" t="n">
+      <c r="AD2" s="1" t="n">
         <v>46094.6985306713</v>
       </c>
       <c r="AE2" t="inlineStr"/>
@@ -775,7 +763,7 @@
           <t>Notificación personal medio electrónico</t>
         </is>
       </c>
-      <c r="L3" s="2" t="n">
+      <c r="L3" s="1" t="n">
         <v>46094.4726014699</v>
       </c>
       <c r="M3" t="inlineStr">
@@ -807,7 +795,7 @@
       <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="inlineStr"/>
       <c r="AC3" t="inlineStr"/>
-      <c r="AD3" s="2" t="n">
+      <c r="AD3" s="1" t="n">
         <v>46094.4726014699</v>
       </c>
       <c r="AE3" t="inlineStr"/>
@@ -885,7 +873,7 @@
           <t>Se hace un Requerimiento</t>
         </is>
       </c>
-      <c r="L4" s="2" t="n">
+      <c r="L4" s="1" t="n">
         <v>46083.90121315972</v>
       </c>
       <c r="M4" t="inlineStr"/>
@@ -909,7 +897,7 @@
       <c r="AA4" t="inlineStr"/>
       <c r="AB4" t="inlineStr"/>
       <c r="AC4" t="inlineStr"/>
-      <c r="AD4" s="2" t="n">
+      <c r="AD4" s="1" t="n">
         <v>46083.90121315972</v>
       </c>
       <c r="AE4" t="inlineStr"/>
@@ -983,7 +971,7 @@
           <t>Declara el Cumplimiento de Unas Obligaciones</t>
         </is>
       </c>
-      <c r="L5" s="2" t="n">
+      <c r="L5" s="1" t="n">
         <v>46099.44996605324</v>
       </c>
       <c r="M5" t="inlineStr"/>
@@ -1007,7 +995,7 @@
       <c r="AA5" t="inlineStr"/>
       <c r="AB5" t="inlineStr"/>
       <c r="AC5" t="inlineStr"/>
-      <c r="AD5" s="2" t="n">
+      <c r="AD5" s="1" t="n">
         <v>46099.44996605324</v>
       </c>
       <c r="AE5" t="inlineStr"/>
@@ -1081,7 +1069,7 @@
           <t>Requerimientos</t>
         </is>
       </c>
-      <c r="L6" s="2" t="n">
+      <c r="L6" s="1" t="n">
         <v>46098.50233163194</v>
       </c>
       <c r="M6" t="inlineStr"/>
@@ -1105,7 +1093,7 @@
       <c r="AA6" t="inlineStr"/>
       <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="inlineStr"/>
-      <c r="AD6" s="2" t="n">
+      <c r="AD6" s="1" t="n">
         <v>46098.50233163194</v>
       </c>
       <c r="AE6" t="inlineStr"/>
@@ -1179,7 +1167,7 @@
           <t>Requerimientos</t>
         </is>
       </c>
-      <c r="L7" s="2" t="n">
+      <c r="L7" s="1" t="n">
         <v>46098.45814351852</v>
       </c>
       <c r="M7" t="inlineStr"/>
@@ -1203,7 +1191,7 @@
       <c r="AA7" t="inlineStr"/>
       <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="inlineStr"/>
-      <c r="AD7" s="2" t="n">
+      <c r="AD7" s="1" t="n">
         <v>46098.45814351852</v>
       </c>
       <c r="AE7" t="inlineStr"/>
@@ -1277,7 +1265,7 @@
           <t>Anuncia de caducidad y realiza cobro por Seguimiento Ambiental</t>
         </is>
       </c>
-      <c r="L8" s="2" t="n">
+      <c r="L8" s="1" t="n">
         <v>46077.4419290162</v>
       </c>
       <c r="M8" t="inlineStr"/>
@@ -1301,7 +1289,7 @@
       <c r="AA8" t="inlineStr"/>
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr"/>
-      <c r="AD8" s="2" t="n">
+      <c r="AD8" s="1" t="n">
         <v>46077.4419290162</v>
       </c>
       <c r="AE8" t="inlineStr"/>
@@ -1375,7 +1363,7 @@
           <t>Requerimientos</t>
         </is>
       </c>
-      <c r="L9" s="2" t="n">
+      <c r="L9" s="1" t="n">
         <v>46078.51178321759</v>
       </c>
       <c r="M9" t="inlineStr"/>
@@ -1399,7 +1387,7 @@
       <c r="AA9" t="inlineStr"/>
       <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr"/>
-      <c r="AD9" s="2" t="n">
+      <c r="AD9" s="1" t="n">
         <v>46078.51178321759</v>
       </c>
       <c r="AE9" t="inlineStr"/>
@@ -1473,7 +1461,7 @@
           <t>Requerimientos</t>
         </is>
       </c>
-      <c r="L10" s="2" t="n">
+      <c r="L10" s="1" t="n">
         <v>46077.51255096065</v>
       </c>
       <c r="M10" t="inlineStr"/>
@@ -1497,7 +1485,7 @@
       <c r="AA10" t="inlineStr"/>
       <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="inlineStr"/>
-      <c r="AD10" s="2" t="n">
+      <c r="AD10" s="1" t="n">
         <v>46077.51255096065</v>
       </c>
       <c r="AE10" t="inlineStr"/>
@@ -1571,7 +1559,7 @@
           <t>Requerimiento y realiza cobro por seguimiento ambiental</t>
         </is>
       </c>
-      <c r="L11" s="2" t="n">
+      <c r="L11" s="1" t="n">
         <v>46077.46326153935</v>
       </c>
       <c r="M11" t="inlineStr"/>
@@ -1595,7 +1583,7 @@
       <c r="AA11" t="inlineStr"/>
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr"/>
-      <c r="AD11" s="2" t="n">
+      <c r="AD11" s="1" t="n">
         <v>46077.46326153935</v>
       </c>
       <c r="AE11" t="inlineStr"/>
@@ -1669,7 +1657,7 @@
           <t>Requerimiento y realiza cobro por seguimiento ambiental</t>
         </is>
       </c>
-      <c r="L12" s="2" t="n">
+      <c r="L12" s="1" t="n">
         <v>46071.37778148148</v>
       </c>
       <c r="M12" t="inlineStr"/>
@@ -1693,7 +1681,7 @@
       <c r="AA12" t="inlineStr"/>
       <c r="AB12" t="inlineStr"/>
       <c r="AC12" t="inlineStr"/>
-      <c r="AD12" s="2" t="n">
+      <c r="AD12" s="1" t="n">
         <v>46071.37778148148</v>
       </c>
       <c r="AE12" t="inlineStr"/>
@@ -1767,7 +1755,7 @@
           <t>Declara la pérdida de fuerza ejecutoria de una resolución</t>
         </is>
       </c>
-      <c r="L13" s="2" t="n">
+      <c r="L13" s="1" t="n">
         <v>46075.93244664352</v>
       </c>
       <c r="M13" t="inlineStr"/>
@@ -1791,7 +1779,7 @@
       <c r="AA13" t="inlineStr"/>
       <c r="AB13" t="inlineStr"/>
       <c r="AC13" t="inlineStr"/>
-      <c r="AD13" s="2" t="n">
+      <c r="AD13" s="1" t="n">
         <v>46075.93244664352</v>
       </c>
       <c r="AE13" t="inlineStr"/>
@@ -1865,7 +1853,7 @@
           <t>Requerimiento y realiza cobro por seguimiento ambiental</t>
         </is>
       </c>
-      <c r="L14" s="2" t="n">
+      <c r="L14" s="1" t="n">
         <v>46075.85217986111</v>
       </c>
       <c r="M14" t="inlineStr"/>
@@ -1889,7 +1877,7 @@
       <c r="AA14" t="inlineStr"/>
       <c r="AB14" t="inlineStr"/>
       <c r="AC14" t="inlineStr"/>
-      <c r="AD14" s="2" t="n">
+      <c r="AD14" s="1" t="n">
         <v>46075.85217986111</v>
       </c>
       <c r="AE14" t="inlineStr"/>
@@ -1963,7 +1951,7 @@
           <t>Exoneración de cobro de evaluación y/o seguimiento</t>
         </is>
       </c>
-      <c r="L15" s="2" t="n">
+      <c r="L15" s="1" t="n">
         <v>46104.79661979167</v>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -1987,7 +1975,7 @@
       <c r="AA15" t="inlineStr"/>
       <c r="AB15" t="inlineStr"/>
       <c r="AC15" t="inlineStr"/>
-      <c r="AD15" s="2" t="n">
+      <c r="AD15" s="1" t="n">
         <v>46104.79661979167</v>
       </c>
       <c r="AE15" t="inlineStr"/>
@@ -2061,7 +2049,7 @@
           <t>Cobro</t>
         </is>
       </c>
-      <c r="L16" s="2" t="n">
+      <c r="L16" s="1" t="n">
         <v>46088.36844780092</v>
       </c>
       <c r="M16" t="inlineStr"/>
@@ -2085,7 +2073,7 @@
       <c r="AA16" t="inlineStr"/>
       <c r="AB16" t="inlineStr"/>
       <c r="AC16" t="inlineStr"/>
-      <c r="AD16" s="2" t="n">
+      <c r="AD16" s="1" t="n">
         <v>46088.36844780092</v>
       </c>
       <c r="AE16" t="inlineStr"/>
@@ -2159,7 +2147,7 @@
           <t>Requerimientos</t>
         </is>
       </c>
-      <c r="L17" s="2" t="n">
+      <c r="L17" s="1" t="n">
         <v>46093.62659355324</v>
       </c>
       <c r="M17" t="inlineStr"/>
@@ -2183,7 +2171,7 @@
       <c r="AA17" t="inlineStr"/>
       <c r="AB17" t="inlineStr"/>
       <c r="AC17" t="inlineStr"/>
-      <c r="AD17" s="2" t="n">
+      <c r="AD17" s="1" t="n">
         <v>46093.62659355324</v>
       </c>
       <c r="AE17" t="inlineStr"/>
@@ -2257,7 +2245,7 @@
           <t>Cobro</t>
         </is>
       </c>
-      <c r="L18" s="2" t="n">
+      <c r="L18" s="1" t="n">
         <v>46088.43574262731</v>
       </c>
       <c r="M18" t="inlineStr"/>
@@ -2281,7 +2269,7 @@
       <c r="AA18" t="inlineStr"/>
       <c r="AB18" t="inlineStr"/>
       <c r="AC18" t="inlineStr"/>
-      <c r="AD18" s="2" t="n">
+      <c r="AD18" s="1" t="n">
         <v>46088.43574262731</v>
       </c>
       <c r="AE18" t="inlineStr"/>
@@ -2355,7 +2343,7 @@
           <t>Exoneración de cobro de evaluación y/o seguimiento</t>
         </is>
       </c>
-      <c r="L19" s="2" t="n">
+      <c r="L19" s="1" t="n">
         <v>46104.34150170139</v>
       </c>
       <c r="M19" t="inlineStr"/>
@@ -2379,7 +2367,7 @@
       <c r="AA19" t="inlineStr"/>
       <c r="AB19" t="inlineStr"/>
       <c r="AC19" t="inlineStr"/>
-      <c r="AD19" s="2" t="n">
+      <c r="AD19" s="1" t="n">
         <v>46104.34150170139</v>
       </c>
       <c r="AE19" t="inlineStr"/>
@@ -2453,7 +2441,7 @@
           <t>Requerimientos</t>
         </is>
       </c>
-      <c r="L20" s="2" t="n">
+      <c r="L20" s="1" t="n">
         <v>46084.61792511574</v>
       </c>
       <c r="M20" t="inlineStr"/>
@@ -2477,7 +2465,7 @@
       <c r="AA20" t="inlineStr"/>
       <c r="AB20" t="inlineStr"/>
       <c r="AC20" t="inlineStr"/>
-      <c r="AD20" s="2" t="n">
+      <c r="AD20" s="1" t="n">
         <v>46084.61792511574</v>
       </c>
       <c r="AE20" t="inlineStr"/>
@@ -2551,7 +2539,7 @@
           <t>Anuncia Caducidad Administrativa C.A. Superficiales</t>
         </is>
       </c>
-      <c r="L21" s="2" t="n">
+      <c r="L21" s="1" t="n">
         <v>46091.75663668982</v>
       </c>
       <c r="M21" t="inlineStr"/>
@@ -2575,7 +2563,7 @@
       <c r="AA21" t="inlineStr"/>
       <c r="AB21" t="inlineStr"/>
       <c r="AC21" t="inlineStr"/>
-      <c r="AD21" s="2" t="n">
+      <c r="AD21" s="1" t="n">
         <v>46091.75663668982</v>
       </c>
       <c r="AE21" t="inlineStr"/>
@@ -2649,7 +2637,7 @@
           <t>Ordena Desarchivo de Un Expediente</t>
         </is>
       </c>
-      <c r="L22" s="2" t="n">
+      <c r="L22" s="1" t="n">
         <v>46098.71219270834</v>
       </c>
       <c r="M22" t="inlineStr"/>
@@ -2673,7 +2661,7 @@
       <c r="AA22" t="inlineStr"/>
       <c r="AB22" t="inlineStr"/>
       <c r="AC22" t="inlineStr"/>
-      <c r="AD22" s="2" t="n">
+      <c r="AD22" s="1" t="n">
         <v>46098.71219270834</v>
       </c>
       <c r="AE22" t="inlineStr"/>
@@ -2747,7 +2735,7 @@
           <t>Por el cual ordena el Archivo de un expediente</t>
         </is>
       </c>
-      <c r="L23" s="2" t="n">
+      <c r="L23" s="1" t="n">
         <v>46100.63619001157</v>
       </c>
       <c r="M23" t="inlineStr"/>
@@ -2771,7 +2759,7 @@
       <c r="AA23" t="inlineStr"/>
       <c r="AB23" t="inlineStr"/>
       <c r="AC23" t="inlineStr"/>
-      <c r="AD23" s="2" t="n">
+      <c r="AD23" s="1" t="n">
         <v>46100.63619001157</v>
       </c>
       <c r="AE23" t="inlineStr"/>
@@ -2845,7 +2833,7 @@
           <t>Exoneración de cobro de evaluación y/o seguimiento</t>
         </is>
       </c>
-      <c r="L24" s="2" t="n">
+      <c r="L24" s="1" t="n">
         <v>46101.86146828704</v>
       </c>
       <c r="M24" t="inlineStr"/>
@@ -2869,7 +2857,7 @@
       <c r="AA24" t="inlineStr"/>
       <c r="AB24" t="inlineStr"/>
       <c r="AC24" t="inlineStr"/>
-      <c r="AD24" s="2" t="n">
+      <c r="AD24" s="1" t="n">
         <v>46101.86146828704</v>
       </c>
       <c r="AE24" t="inlineStr"/>
@@ -2943,7 +2931,7 @@
           <t>Cobro</t>
         </is>
       </c>
-      <c r="L25" s="2" t="n">
+      <c r="L25" s="1" t="n">
         <v>46087.95318989583</v>
       </c>
       <c r="M25" t="inlineStr"/>
@@ -2967,7 +2955,7 @@
       <c r="AA25" t="inlineStr"/>
       <c r="AB25" t="inlineStr"/>
       <c r="AC25" t="inlineStr"/>
-      <c r="AD25" s="2" t="n">
+      <c r="AD25" s="1" t="n">
         <v>46087.95318989583</v>
       </c>
       <c r="AE25" t="inlineStr"/>
@@ -3041,7 +3029,7 @@
           <t>Cobro</t>
         </is>
       </c>
-      <c r="L26" s="2" t="n">
+      <c r="L26" s="1" t="n">
         <v>46087.38717071759</v>
       </c>
       <c r="M26" t="inlineStr"/>
@@ -3065,7 +3053,7 @@
       <c r="AA26" t="inlineStr"/>
       <c r="AB26" t="inlineStr"/>
       <c r="AC26" t="inlineStr"/>
-      <c r="AD26" s="2" t="n">
+      <c r="AD26" s="1" t="n">
         <v>46087.38717071759</v>
       </c>
       <c r="AE26" t="inlineStr"/>
@@ -3139,7 +3127,7 @@
           <t>Cobro</t>
         </is>
       </c>
-      <c r="L27" s="2" t="n">
+      <c r="L27" s="1" t="n">
         <v>46086.81106111111</v>
       </c>
       <c r="M27" t="inlineStr"/>
@@ -3163,7 +3151,7 @@
       <c r="AA27" t="inlineStr"/>
       <c r="AB27" t="inlineStr"/>
       <c r="AC27" t="inlineStr"/>
-      <c r="AD27" s="2" t="n">
+      <c r="AD27" s="1" t="n">
         <v>46086.81106111111</v>
       </c>
       <c r="AE27" t="inlineStr"/>
@@ -3237,7 +3225,7 @@
           <t>Cobro</t>
         </is>
       </c>
-      <c r="L28" s="2" t="n">
+      <c r="L28" s="1" t="n">
         <v>46085.69307418982</v>
       </c>
       <c r="M28" t="inlineStr"/>
@@ -3261,7 +3249,7 @@
       <c r="AA28" t="inlineStr"/>
       <c r="AB28" t="inlineStr"/>
       <c r="AC28" t="inlineStr"/>
-      <c r="AD28" s="2" t="n">
+      <c r="AD28" s="1" t="n">
         <v>46085.69307418982</v>
       </c>
       <c r="AE28" t="inlineStr"/>
@@ -3335,7 +3323,7 @@
           <t>Cobro</t>
         </is>
       </c>
-      <c r="L29" s="2" t="n">
+      <c r="L29" s="1" t="n">
         <v>46079.73432855324</v>
       </c>
       <c r="M29" t="inlineStr"/>
@@ -3359,7 +3347,7 @@
       <c r="AA29" t="inlineStr"/>
       <c r="AB29" t="inlineStr"/>
       <c r="AC29" t="inlineStr"/>
-      <c r="AD29" s="2" t="n">
+      <c r="AD29" s="1" t="n">
         <v>46079.73432855324</v>
       </c>
       <c r="AE29" t="inlineStr"/>
@@ -3433,7 +3421,7 @@
           <t>Cobro</t>
         </is>
       </c>
-      <c r="L30" s="2" t="n">
+      <c r="L30" s="1" t="n">
         <v>46081.4726658912</v>
       </c>
       <c r="M30" t="inlineStr"/>
@@ -3457,7 +3445,7 @@
       <c r="AA30" t="inlineStr"/>
       <c r="AB30" t="inlineStr"/>
       <c r="AC30" t="inlineStr"/>
-      <c r="AD30" s="2" t="n">
+      <c r="AD30" s="1" t="n">
         <v>46081.4726658912</v>
       </c>
       <c r="AE30" t="inlineStr"/>
@@ -3531,7 +3519,7 @@
           <t>Aprueba un programa de uso eficiente y ahorro de agua</t>
         </is>
       </c>
-      <c r="L31" s="2" t="n">
+      <c r="L31" s="1" t="n">
         <v>46079.51011180555</v>
       </c>
       <c r="M31" t="inlineStr"/>
@@ -3555,7 +3543,7 @@
       <c r="AA31" t="inlineStr"/>
       <c r="AB31" t="inlineStr"/>
       <c r="AC31" t="inlineStr"/>
-      <c r="AD31" s="2" t="n">
+      <c r="AD31" s="1" t="n">
         <v>46079.51011180555</v>
       </c>
       <c r="AE31" t="inlineStr"/>
@@ -3629,7 +3617,7 @@
           <t>Cobro</t>
         </is>
       </c>
-      <c r="L32" s="2" t="n">
+      <c r="L32" s="1" t="n">
         <v>46079.6516383912</v>
       </c>
       <c r="M32" t="inlineStr"/>
@@ -3653,7 +3641,7 @@
       <c r="AA32" t="inlineStr"/>
       <c r="AB32" t="inlineStr"/>
       <c r="AC32" t="inlineStr"/>
-      <c r="AD32" s="2" t="n">
+      <c r="AD32" s="1" t="n">
         <v>46079.6516383912</v>
       </c>
       <c r="AE32" t="inlineStr"/>
@@ -3732,7 +3720,7 @@
           <t>Enviado para Revisión</t>
         </is>
       </c>
-      <c r="S33" s="2" t="n">
+      <c r="S33" s="1" t="n">
         <v>46076.50913116898</v>
       </c>
       <c r="T33" t="inlineStr">
@@ -3751,7 +3739,7 @@
       <c r="AA33" t="inlineStr"/>
       <c r="AB33" t="inlineStr"/>
       <c r="AC33" t="inlineStr"/>
-      <c r="AD33" s="2" t="n">
+      <c r="AD33" s="1" t="n">
         <v>46076.50913116898</v>
       </c>
       <c r="AE33" t="inlineStr"/>
@@ -3825,7 +3813,7 @@
           <t>Cobro</t>
         </is>
       </c>
-      <c r="L34" s="2" t="n">
+      <c r="L34" s="1" t="n">
         <v>46076.69752075231</v>
       </c>
       <c r="M34" t="inlineStr"/>
@@ -3849,7 +3837,7 @@
       <c r="AA34" t="inlineStr"/>
       <c r="AB34" t="inlineStr"/>
       <c r="AC34" t="inlineStr"/>
-      <c r="AD34" s="2" t="n">
+      <c r="AD34" s="1" t="n">
         <v>46076.69752075231</v>
       </c>
       <c r="AE34" t="inlineStr"/>
@@ -3923,7 +3911,7 @@
           <t>Cobro</t>
         </is>
       </c>
-      <c r="L35" s="2" t="n">
+      <c r="L35" s="1" t="n">
         <v>46076.70917670139</v>
       </c>
       <c r="M35" t="inlineStr"/>
@@ -3947,7 +3935,7 @@
       <c r="AA35" t="inlineStr"/>
       <c r="AB35" t="inlineStr"/>
       <c r="AC35" t="inlineStr"/>
-      <c r="AD35" s="2" t="n">
+      <c r="AD35" s="1" t="n">
         <v>46076.70917670139</v>
       </c>
       <c r="AE35" t="inlineStr"/>
@@ -4021,7 +4009,7 @@
           <t>Cobro</t>
         </is>
       </c>
-      <c r="L36" s="2" t="n">
+      <c r="L36" s="1" t="n">
         <v>46076.7546</v>
       </c>
       <c r="M36" t="inlineStr"/>
@@ -4045,7 +4033,7 @@
       <c r="AA36" t="inlineStr"/>
       <c r="AB36" t="inlineStr"/>
       <c r="AC36" t="inlineStr"/>
-      <c r="AD36" s="2" t="n">
+      <c r="AD36" s="1" t="n">
         <v>46076.7546</v>
       </c>
       <c r="AE36" t="inlineStr"/>
@@ -4119,7 +4107,7 @@
           <t>Anuncia de caducidad y realiza cobro por Seguimiento Ambiental</t>
         </is>
       </c>
-      <c r="L37" s="2" t="n">
+      <c r="L37" s="1" t="n">
         <v>46099.93035486111</v>
       </c>
       <c r="M37" t="inlineStr">
@@ -4150,7 +4138,7 @@
           <t>Enviado para Revisión</t>
         </is>
       </c>
-      <c r="S37" s="2" t="n">
+      <c r="S37" s="1" t="n">
         <v>46105.42905096065</v>
       </c>
       <c r="T37" t="inlineStr">
@@ -4169,7 +4157,7 @@
       <c r="AA37" t="inlineStr"/>
       <c r="AB37" t="inlineStr"/>
       <c r="AC37" t="inlineStr"/>
-      <c r="AD37" s="2" t="n">
+      <c r="AD37" s="1" t="n">
         <v>46105.42905096065</v>
       </c>
       <c r="AE37" t="inlineStr"/>
@@ -4247,7 +4235,7 @@
           <t>Cobro</t>
         </is>
       </c>
-      <c r="L38" s="2" t="n">
+      <c r="L38" s="1" t="n">
         <v>46098.93157311343</v>
       </c>
       <c r="M38" t="inlineStr">
@@ -4278,7 +4266,7 @@
           <t>Enviado para Revisión</t>
         </is>
       </c>
-      <c r="S38" s="2" t="n">
+      <c r="S38" s="1" t="n">
         <v>46105.4854053588</v>
       </c>
       <c r="T38" t="inlineStr">
@@ -4297,7 +4285,7 @@
       <c r="AA38" t="inlineStr"/>
       <c r="AB38" t="inlineStr"/>
       <c r="AC38" t="inlineStr"/>
-      <c r="AD38" s="2" t="n">
+      <c r="AD38" s="1" t="n">
         <v>46105.4854053588</v>
       </c>
       <c r="AE38" t="inlineStr"/>
@@ -4375,7 +4363,7 @@
           <t>Anuncia de caducidad y realiza cobro por Seguimiento Ambiental</t>
         </is>
       </c>
-      <c r="L39" s="2" t="n">
+      <c r="L39" s="1" t="n">
         <v>46099.90207769676</v>
       </c>
       <c r="M39" t="inlineStr">
@@ -4406,7 +4394,7 @@
           <t>Enviado para Revisión</t>
         </is>
       </c>
-      <c r="S39" s="2" t="n">
+      <c r="S39" s="1" t="n">
         <v>46105.47745940973</v>
       </c>
       <c r="T39" t="inlineStr">
@@ -4425,7 +4413,7 @@
       <c r="AA39" t="inlineStr"/>
       <c r="AB39" t="inlineStr"/>
       <c r="AC39" t="inlineStr"/>
-      <c r="AD39" s="2" t="n">
+      <c r="AD39" s="1" t="n">
         <v>46105.47745940973</v>
       </c>
       <c r="AE39" t="inlineStr"/>
@@ -4503,7 +4491,7 @@
           <t>Requerimiento y realiza cobro por seguimiento ambiental</t>
         </is>
       </c>
-      <c r="L40" s="2" t="n">
+      <c r="L40" s="1" t="n">
         <v>46097.46426056713</v>
       </c>
       <c r="M40" t="inlineStr"/>
@@ -4527,7 +4515,7 @@
       <c r="AA40" t="inlineStr"/>
       <c r="AB40" t="inlineStr"/>
       <c r="AC40" t="inlineStr"/>
-      <c r="AD40" s="2" t="n">
+      <c r="AD40" s="1" t="n">
         <v>46097.46426056713</v>
       </c>
       <c r="AE40" t="inlineStr"/>
@@ -4601,7 +4589,7 @@
           <t>Requerimiento y realiza cobro por seguimiento ambiental</t>
         </is>
       </c>
-      <c r="L41" s="2" t="n">
+      <c r="L41" s="1" t="n">
         <v>46101.79273788194</v>
       </c>
       <c r="M41" t="inlineStr"/>
@@ -4625,7 +4613,7 @@
       <c r="AA41" t="inlineStr"/>
       <c r="AB41" t="inlineStr"/>
       <c r="AC41" t="inlineStr"/>
-      <c r="AD41" s="2" t="n">
+      <c r="AD41" s="1" t="n">
         <v>46101.79273788194</v>
       </c>
       <c r="AE41" t="inlineStr"/>
@@ -4699,7 +4687,7 @@
           <t>Requerimientos</t>
         </is>
       </c>
-      <c r="L42" s="2" t="n">
+      <c r="L42" s="1" t="n">
         <v>46101.80057195602</v>
       </c>
       <c r="M42" t="inlineStr"/>
@@ -4723,7 +4711,7 @@
       <c r="AA42" t="inlineStr"/>
       <c r="AB42" t="inlineStr"/>
       <c r="AC42" t="inlineStr"/>
-      <c r="AD42" s="2" t="n">
+      <c r="AD42" s="1" t="n">
         <v>46101.80057195602</v>
       </c>
       <c r="AE42" t="inlineStr"/>
@@ -4797,7 +4785,7 @@
           <t>Declara la pérdida de fuerza ejecutoria de una resolución</t>
         </is>
       </c>
-      <c r="L43" s="2" t="n">
+      <c r="L43" s="1" t="n">
         <v>46092.47107623843</v>
       </c>
       <c r="M43" t="inlineStr">
@@ -4829,7 +4817,7 @@
       <c r="AA43" t="inlineStr"/>
       <c r="AB43" t="inlineStr"/>
       <c r="AC43" t="inlineStr"/>
-      <c r="AD43" s="2" t="n">
+      <c r="AD43" s="1" t="n">
         <v>46092.47107623843</v>
       </c>
       <c r="AE43" t="inlineStr"/>
@@ -4907,7 +4895,7 @@
           <t>PUEAA - APRUEBA Programa de Uso Eficiente y Ahorro de Agua</t>
         </is>
       </c>
-      <c r="L44" s="2" t="n">
+      <c r="L44" s="1" t="n">
         <v>46101.80507318287</v>
       </c>
       <c r="M44" t="inlineStr"/>
@@ -4931,7 +4919,7 @@
       <c r="AA44" t="inlineStr"/>
       <c r="AB44" t="inlineStr"/>
       <c r="AC44" t="inlineStr"/>
-      <c r="AD44" s="2" t="n">
+      <c r="AD44" s="1" t="n">
         <v>46101.80507318287</v>
       </c>
       <c r="AE44" t="inlineStr"/>
@@ -5005,7 +4993,7 @@
           <t>Anuncia de caducidad y realiza cobro por Seguimiento Ambiental</t>
         </is>
       </c>
-      <c r="L45" s="2" t="n">
+      <c r="L45" s="1" t="n">
         <v>46097.67375424768</v>
       </c>
       <c r="M45" t="inlineStr">
@@ -5037,7 +5025,7 @@
       <c r="AA45" t="inlineStr"/>
       <c r="AB45" t="inlineStr"/>
       <c r="AC45" t="inlineStr"/>
-      <c r="AD45" s="2" t="n">
+      <c r="AD45" s="1" t="n">
         <v>46097.67375424768</v>
       </c>
       <c r="AE45" t="inlineStr"/>
@@ -5115,7 +5103,7 @@
           <t>Cobro</t>
         </is>
       </c>
-      <c r="L46" s="2" t="n">
+      <c r="L46" s="1" t="n">
         <v>46097.67692546296</v>
       </c>
       <c r="M46" t="inlineStr">
@@ -5147,7 +5135,7 @@
       <c r="AA46" t="inlineStr"/>
       <c r="AB46" t="inlineStr"/>
       <c r="AC46" t="inlineStr"/>
-      <c r="AD46" s="2" t="n">
+      <c r="AD46" s="1" t="n">
         <v>46097.67692546296</v>
       </c>
       <c r="AE46" t="inlineStr"/>
@@ -5225,7 +5213,7 @@
           <t>Requerimiento y realiza cobro por seguimiento ambiental</t>
         </is>
       </c>
-      <c r="L47" s="2" t="n">
+      <c r="L47" s="1" t="n">
         <v>46105.38046061343</v>
       </c>
       <c r="M47" t="inlineStr"/>
@@ -5249,7 +5237,7 @@
       <c r="AA47" t="inlineStr"/>
       <c r="AB47" t="inlineStr"/>
       <c r="AC47" t="inlineStr"/>
-      <c r="AD47" s="2" t="n">
+      <c r="AD47" s="1" t="n">
         <v>46105.38046061343</v>
       </c>
       <c r="AE47" t="inlineStr"/>
@@ -5323,7 +5311,7 @@
           <t>Requerimiento y realiza cobro por seguimiento ambiental</t>
         </is>
       </c>
-      <c r="L48" s="2" t="n">
+      <c r="L48" s="1" t="n">
         <v>46097.49573973379</v>
       </c>
       <c r="M48" t="inlineStr"/>
@@ -5347,7 +5335,7 @@
       <c r="AA48" t="inlineStr"/>
       <c r="AB48" t="inlineStr"/>
       <c r="AC48" t="inlineStr"/>
-      <c r="AD48" s="2" t="n">
+      <c r="AD48" s="1" t="n">
         <v>46097.49573973379</v>
       </c>
       <c r="AE48" t="inlineStr"/>
@@ -5421,7 +5409,7 @@
           <t>Anuncia de caducidad y realiza cobro por Seguimiento Ambiental</t>
         </is>
       </c>
-      <c r="L49" s="2" t="n">
+      <c r="L49" s="1" t="n">
         <v>46099.93246898148</v>
       </c>
       <c r="M49" t="inlineStr">
@@ -5453,7 +5441,7 @@
       <c r="AA49" t="inlineStr"/>
       <c r="AB49" t="inlineStr"/>
       <c r="AC49" t="inlineStr"/>
-      <c r="AD49" s="2" t="n">
+      <c r="AD49" s="1" t="n">
         <v>46099.93246898148</v>
       </c>
       <c r="AE49" t="inlineStr"/>
@@ -5531,7 +5519,7 @@
           <t>Requerimiento y realiza cobro por seguimiento ambiental</t>
         </is>
       </c>
-      <c r="L50" s="2" t="n">
+      <c r="L50" s="1" t="n">
         <v>46097.49147129629</v>
       </c>
       <c r="M50" t="inlineStr"/>
@@ -5555,7 +5543,7 @@
       <c r="AA50" t="inlineStr"/>
       <c r="AB50" t="inlineStr"/>
       <c r="AC50" t="inlineStr"/>
-      <c r="AD50" s="2" t="n">
+      <c r="AD50" s="1" t="n">
         <v>46097.49147129629</v>
       </c>
       <c r="AE50" t="inlineStr"/>
@@ -5629,7 +5617,7 @@
           <t>Anuncia de caducidad y realiza cobro por Seguimiento Ambiental</t>
         </is>
       </c>
-      <c r="L51" s="2" t="n">
+      <c r="L51" s="1" t="n">
         <v>46083.84801006944</v>
       </c>
       <c r="M51" t="inlineStr"/>
@@ -5653,7 +5641,7 @@
       <c r="AA51" t="inlineStr"/>
       <c r="AB51" t="inlineStr"/>
       <c r="AC51" t="inlineStr"/>
-      <c r="AD51" s="2" t="n">
+      <c r="AD51" s="1" t="n">
         <v>46083.84801006944</v>
       </c>
       <c r="AE51" t="inlineStr"/>
@@ -5727,7 +5715,7 @@
           <t>Declara la pérdida de fuerza ejecutoria de una resolución</t>
         </is>
       </c>
-      <c r="L52" s="2" t="n">
+      <c r="L52" s="1" t="n">
         <v>46098.42446840278</v>
       </c>
       <c r="M52" t="inlineStr">
@@ -5767,7 +5755,7 @@
           <t>Radicado</t>
         </is>
       </c>
-      <c r="Z52" s="2" t="n">
+      <c r="Z52" s="1" t="n">
         <v>46098.42446840278</v>
       </c>
       <c r="AA52" t="inlineStr">
@@ -5785,10 +5773,10 @@
           <t>Alvaro Andres Jimenez Vanegas / DJA, Andres Mauricio Garzón Orjuela / DRSC</t>
         </is>
       </c>
-      <c r="AD52" s="2" t="n">
+      <c r="AD52" s="1" t="n">
         <v>46098.42446840278</v>
       </c>
-      <c r="AE52" s="2" t="n">
+      <c r="AE52" s="1" t="n">
         <v>46098.42446840278</v>
       </c>
       <c r="AF52" t="n">
@@ -5865,7 +5853,7 @@
           <t>PUEAA - APRUEBA Programa de Uso Eficiente y Ahorro de Agua</t>
         </is>
       </c>
-      <c r="L53" s="2" t="n">
+      <c r="L53" s="1" t="n">
         <v>46080.40955185185</v>
       </c>
       <c r="M53" t="inlineStr">
@@ -5897,7 +5885,7 @@
       <c r="AA53" t="inlineStr"/>
       <c r="AB53" t="inlineStr"/>
       <c r="AC53" t="inlineStr"/>
-      <c r="AD53" s="2" t="n">
+      <c r="AD53" s="1" t="n">
         <v>46080.40955185185</v>
       </c>
       <c r="AE53" t="inlineStr"/>
@@ -5975,7 +5963,7 @@
           <t>Cobro</t>
         </is>
       </c>
-      <c r="L54" s="2" t="n">
+      <c r="L54" s="1" t="n">
         <v>46077.48910193287</v>
       </c>
       <c r="M54" t="inlineStr"/>
@@ -5999,7 +5987,7 @@
       <c r="AA54" t="inlineStr"/>
       <c r="AB54" t="inlineStr"/>
       <c r="AC54" t="inlineStr"/>
-      <c r="AD54" s="2" t="n">
+      <c r="AD54" s="1" t="n">
         <v>46077.48910193287</v>
       </c>
       <c r="AE54" t="inlineStr"/>
@@ -6073,7 +6061,7 @@
           <t>PUEAA - APRUEBA Programa de Uso Eficiente y Ahorro de Agua</t>
         </is>
       </c>
-      <c r="L55" s="2" t="n">
+      <c r="L55" s="1" t="n">
         <v>46079.31786215278</v>
       </c>
       <c r="M55" t="inlineStr">
@@ -6105,7 +6093,7 @@
       <c r="AA55" t="inlineStr"/>
       <c r="AB55" t="inlineStr"/>
       <c r="AC55" t="inlineStr"/>
-      <c r="AD55" s="2" t="n">
+      <c r="AD55" s="1" t="n">
         <v>46079.31786215278</v>
       </c>
       <c r="AE55" t="inlineStr"/>
@@ -6183,7 +6171,7 @@
           <t>Acepta la Renuncia de una Concesión de Aguas Superficiales</t>
         </is>
       </c>
-      <c r="L56" s="2" t="n">
+      <c r="L56" s="1" t="n">
         <v>46077.62005181713</v>
       </c>
       <c r="M56" t="inlineStr">
@@ -6215,7 +6203,7 @@
       <c r="AA56" t="inlineStr"/>
       <c r="AB56" t="inlineStr"/>
       <c r="AC56" t="inlineStr"/>
-      <c r="AD56" s="2" t="n">
+      <c r="AD56" s="1" t="n">
         <v>46077.62005181713</v>
       </c>
       <c r="AE56" t="inlineStr"/>
@@ -6293,7 +6281,7 @@
           <t>Anuncia Caducidad Administrativa C.A. Superficiales</t>
         </is>
       </c>
-      <c r="L57" s="2" t="n">
+      <c r="L57" s="1" t="n">
         <v>46069.71270185185</v>
       </c>
       <c r="M57" t="inlineStr"/>
@@ -6317,7 +6305,7 @@
       <c r="AA57" t="inlineStr"/>
       <c r="AB57" t="inlineStr"/>
       <c r="AC57" t="inlineStr"/>
-      <c r="AD57" s="2" t="n">
+      <c r="AD57" s="1" t="n">
         <v>46069.71270185185</v>
       </c>
       <c r="AE57" t="inlineStr"/>
@@ -6391,7 +6379,7 @@
           <t>Requerimientos</t>
         </is>
       </c>
-      <c r="L58" s="2" t="n">
+      <c r="L58" s="1" t="n">
         <v>46087.61630447917</v>
       </c>
       <c r="M58" t="inlineStr">
@@ -6423,7 +6411,7 @@
       <c r="AA58" t="inlineStr"/>
       <c r="AB58" t="inlineStr"/>
       <c r="AC58" t="inlineStr"/>
-      <c r="AD58" s="2" t="n">
+      <c r="AD58" s="1" t="n">
         <v>46087.61630447917</v>
       </c>
       <c r="AE58" t="inlineStr"/>
@@ -6501,7 +6489,7 @@
           <t>Requerimientos</t>
         </is>
       </c>
-      <c r="L59" s="2" t="n">
+      <c r="L59" s="1" t="n">
         <v>46084.40257133102</v>
       </c>
       <c r="M59" t="inlineStr">
@@ -6533,7 +6521,7 @@
       <c r="AA59" t="inlineStr"/>
       <c r="AB59" t="inlineStr"/>
       <c r="AC59" t="inlineStr"/>
-      <c r="AD59" s="2" t="n">
+      <c r="AD59" s="1" t="n">
         <v>46084.40257133102</v>
       </c>
       <c r="AE59" t="inlineStr"/>
@@ -6611,7 +6599,7 @@
           <t>Requerimientos</t>
         </is>
       </c>
-      <c r="L60" s="2" t="n">
+      <c r="L60" s="1" t="n">
         <v>46086.46862399305</v>
       </c>
       <c r="M60" t="inlineStr">
@@ -6643,7 +6631,7 @@
       <c r="AA60" t="inlineStr"/>
       <c r="AB60" t="inlineStr"/>
       <c r="AC60" t="inlineStr"/>
-      <c r="AD60" s="2" t="n">
+      <c r="AD60" s="1" t="n">
         <v>46086.46862399305</v>
       </c>
       <c r="AE60" t="inlineStr"/>
@@ -6721,7 +6709,7 @@
           <t>Requerimientos</t>
         </is>
       </c>
-      <c r="L61" s="2" t="n">
+      <c r="L61" s="1" t="n">
         <v>46086.37650239583</v>
       </c>
       <c r="M61" t="inlineStr">
@@ -6753,7 +6741,7 @@
       <c r="AA61" t="inlineStr"/>
       <c r="AB61" t="inlineStr"/>
       <c r="AC61" t="inlineStr"/>
-      <c r="AD61" s="2" t="n">
+      <c r="AD61" s="1" t="n">
         <v>46086.37650239583</v>
       </c>
       <c r="AE61" t="inlineStr"/>
@@ -6831,7 +6819,7 @@
           <t>Requerimientos</t>
         </is>
       </c>
-      <c r="L62" s="2" t="n">
+      <c r="L62" s="1" t="n">
         <v>46087.61345277778</v>
       </c>
       <c r="M62" t="inlineStr">
@@ -6863,7 +6851,7 @@
       <c r="AA62" t="inlineStr"/>
       <c r="AB62" t="inlineStr"/>
       <c r="AC62" t="inlineStr"/>
-      <c r="AD62" s="2" t="n">
+      <c r="AD62" s="1" t="n">
         <v>46087.61345277778</v>
       </c>
       <c r="AE62" t="inlineStr"/>
@@ -6941,7 +6929,7 @@
           <t>Requerimientos</t>
         </is>
       </c>
-      <c r="L63" s="2" t="n">
+      <c r="L63" s="1" t="n">
         <v>46087.61262457176</v>
       </c>
       <c r="M63" t="inlineStr">
@@ -6973,7 +6961,7 @@
       <c r="AA63" t="inlineStr"/>
       <c r="AB63" t="inlineStr"/>
       <c r="AC63" t="inlineStr"/>
-      <c r="AD63" s="2" t="n">
+      <c r="AD63" s="1" t="n">
         <v>46087.61262457176</v>
       </c>
       <c r="AE63" t="inlineStr"/>
@@ -7051,7 +7039,7 @@
           <t>Requerimiento y realiza cobro por seguimiento ambiental</t>
         </is>
       </c>
-      <c r="L64" s="2" t="n">
+      <c r="L64" s="1" t="n">
         <v>46087.61520910879</v>
       </c>
       <c r="M64" t="inlineStr">
@@ -7083,7 +7071,7 @@
       <c r="AA64" t="inlineStr"/>
       <c r="AB64" t="inlineStr"/>
       <c r="AC64" t="inlineStr"/>
-      <c r="AD64" s="2" t="n">
+      <c r="AD64" s="1" t="n">
         <v>46087.61520910879</v>
       </c>
       <c r="AE64" t="inlineStr"/>
@@ -7161,7 +7149,7 @@
           <t>Requerimiento y realiza cobro por seguimiento ambiental</t>
         </is>
       </c>
-      <c r="L65" s="2" t="n">
+      <c r="L65" s="1" t="n">
         <v>46083.46959494213</v>
       </c>
       <c r="M65" t="inlineStr"/>
@@ -7185,7 +7173,7 @@
       <c r="AA65" t="inlineStr"/>
       <c r="AB65" t="inlineStr"/>
       <c r="AC65" t="inlineStr"/>
-      <c r="AD65" s="2" t="n">
+      <c r="AD65" s="1" t="n">
         <v>46083.46959494213</v>
       </c>
       <c r="AE65" t="inlineStr"/>
@@ -7259,7 +7247,7 @@
           <t>Requerimiento y realiza cobro por seguimiento ambiental</t>
         </is>
       </c>
-      <c r="L66" s="2" t="n">
+      <c r="L66" s="1" t="n">
         <v>46091.44263680556</v>
       </c>
       <c r="M66" t="inlineStr">
@@ -7291,7 +7279,7 @@
       <c r="AA66" t="inlineStr"/>
       <c r="AB66" t="inlineStr"/>
       <c r="AC66" t="inlineStr"/>
-      <c r="AD66" s="2" t="n">
+      <c r="AD66" s="1" t="n">
         <v>46091.44263680556</v>
       </c>
       <c r="AE66" t="inlineStr"/>
@@ -7369,7 +7357,7 @@
           <t>Requerimientos</t>
         </is>
       </c>
-      <c r="L67" s="2" t="n">
+      <c r="L67" s="1" t="n">
         <v>46086.62741496527</v>
       </c>
       <c r="M67" t="inlineStr">
@@ -7401,7 +7389,7 @@
       <c r="AA67" t="inlineStr"/>
       <c r="AB67" t="inlineStr"/>
       <c r="AC67" t="inlineStr"/>
-      <c r="AD67" s="2" t="n">
+      <c r="AD67" s="1" t="n">
         <v>46086.62741496527</v>
       </c>
       <c r="AE67" t="inlineStr"/>
@@ -7479,7 +7467,7 @@
           <t>Requerimiento y realiza cobro por seguimiento ambiental</t>
         </is>
       </c>
-      <c r="L68" s="2" t="n">
+      <c r="L68" s="1" t="n">
         <v>46091.41339725695</v>
       </c>
       <c r="M68" t="inlineStr">
@@ -7511,7 +7499,7 @@
       <c r="AA68" t="inlineStr"/>
       <c r="AB68" t="inlineStr"/>
       <c r="AC68" t="inlineStr"/>
-      <c r="AD68" s="2" t="n">
+      <c r="AD68" s="1" t="n">
         <v>46091.41339725695</v>
       </c>
       <c r="AE68" t="inlineStr"/>
@@ -7589,7 +7577,7 @@
           <t>Requerimiento y realiza cobro por seguimiento ambiental</t>
         </is>
       </c>
-      <c r="L69" s="2" t="n">
+      <c r="L69" s="1" t="n">
         <v>46091.44262994213</v>
       </c>
       <c r="M69" t="inlineStr">
@@ -7621,7 +7609,7 @@
       <c r="AA69" t="inlineStr"/>
       <c r="AB69" t="inlineStr"/>
       <c r="AC69" t="inlineStr"/>
-      <c r="AD69" s="2" t="n">
+      <c r="AD69" s="1" t="n">
         <v>46091.44262994213</v>
       </c>
       <c r="AE69" t="inlineStr"/>
@@ -7699,7 +7687,7 @@
           <t>Modifica un acto Administrativo</t>
         </is>
       </c>
-      <c r="L70" s="2" t="n">
+      <c r="L70" s="1" t="n">
         <v>46078.59578888889</v>
       </c>
       <c r="M70" t="inlineStr">
@@ -7739,7 +7727,7 @@
           <t>Radicado</t>
         </is>
       </c>
-      <c r="Z70" s="2" t="n">
+      <c r="Z70" s="1" t="n">
         <v>46078.59578888889</v>
       </c>
       <c r="AA70" t="inlineStr">
@@ -7757,10 +7745,10 @@
           <t>Iván Mauricio Castillo Arenas / DJA</t>
         </is>
       </c>
-      <c r="AD70" s="2" t="n">
+      <c r="AD70" s="1" t="n">
         <v>46078.59578888889</v>
       </c>
-      <c r="AE70" s="2" t="n">
+      <c r="AE70" s="1" t="n">
         <v>46078.59578888889</v>
       </c>
       <c r="AF70" t="n">
@@ -7837,7 +7825,7 @@
           <t>Requerimientos</t>
         </is>
       </c>
-      <c r="L71" s="2" t="n">
+      <c r="L71" s="1" t="n">
         <v>46078.54320065973</v>
       </c>
       <c r="M71" t="inlineStr"/>
@@ -7861,7 +7849,7 @@
       <c r="AA71" t="inlineStr"/>
       <c r="AB71" t="inlineStr"/>
       <c r="AC71" t="inlineStr"/>
-      <c r="AD71" s="2" t="n">
+      <c r="AD71" s="1" t="n">
         <v>46078.54320065973</v>
       </c>
       <c r="AE71" t="inlineStr"/>
@@ -7935,7 +7923,7 @@
           <t>Requerimiento y realiza cobro por seguimiento ambiental</t>
         </is>
       </c>
-      <c r="L72" s="2" t="n">
+      <c r="L72" s="1" t="n">
         <v>46079.59924799768</v>
       </c>
       <c r="M72" t="inlineStr"/>
@@ -7959,7 +7947,7 @@
       <c r="AA72" t="inlineStr"/>
       <c r="AB72" t="inlineStr"/>
       <c r="AC72" t="inlineStr"/>
-      <c r="AD72" s="2" t="n">
+      <c r="AD72" s="1" t="n">
         <v>46079.59924799768</v>
       </c>
       <c r="AE72" t="inlineStr"/>
@@ -8033,7 +8021,7 @@
           <t>Requerimientos</t>
         </is>
       </c>
-      <c r="L73" s="2" t="n">
+      <c r="L73" s="1" t="n">
         <v>46079.31656755787</v>
       </c>
       <c r="M73" t="inlineStr">
@@ -8065,7 +8053,7 @@
       <c r="AA73" t="inlineStr"/>
       <c r="AB73" t="inlineStr"/>
       <c r="AC73" t="inlineStr"/>
-      <c r="AD73" s="2" t="n">
+      <c r="AD73" s="1" t="n">
         <v>46079.31656755787</v>
       </c>
       <c r="AE73" t="inlineStr"/>
@@ -8143,7 +8131,7 @@
           <t>Requerimiento y realiza cobro por seguimiento ambiental</t>
         </is>
       </c>
-      <c r="L74" s="2" t="n">
+      <c r="L74" s="1" t="n">
         <v>46079.89292708333</v>
       </c>
       <c r="M74" t="inlineStr">
@@ -8175,7 +8163,7 @@
       <c r="AA74" t="inlineStr"/>
       <c r="AB74" t="inlineStr"/>
       <c r="AC74" t="inlineStr"/>
-      <c r="AD74" s="2" t="n">
+      <c r="AD74" s="1" t="n">
         <v>46079.89292708333</v>
       </c>
       <c r="AE74" t="inlineStr"/>
@@ -8253,7 +8241,7 @@
           <t>Requerimiento y realiza cobro por seguimiento ambiental</t>
         </is>
       </c>
-      <c r="L75" s="2" t="n">
+      <c r="L75" s="1" t="n">
         <v>46079.67824097222</v>
       </c>
       <c r="M75" t="inlineStr">
@@ -8285,7 +8273,7 @@
       <c r="AA75" t="inlineStr"/>
       <c r="AB75" t="inlineStr"/>
       <c r="AC75" t="inlineStr"/>
-      <c r="AD75" s="2" t="n">
+      <c r="AD75" s="1" t="n">
         <v>46079.67824097222</v>
       </c>
       <c r="AE75" t="inlineStr"/>
@@ -8363,7 +8351,7 @@
           <t>Requerimiento y realiza cobro por seguimiento ambiental</t>
         </is>
       </c>
-      <c r="L76" s="2" t="n">
+      <c r="L76" s="1" t="n">
         <v>46077.50019814815</v>
       </c>
       <c r="M76" t="inlineStr">
@@ -8395,7 +8383,7 @@
       <c r="AA76" t="inlineStr"/>
       <c r="AB76" t="inlineStr"/>
       <c r="AC76" t="inlineStr"/>
-      <c r="AD76" s="2" t="n">
+      <c r="AD76" s="1" t="n">
         <v>46077.50019814815</v>
       </c>
       <c r="AE76" t="inlineStr"/>
@@ -8473,7 +8461,7 @@
           <t>Requerimiento y realiza cobro por seguimiento ambiental</t>
         </is>
       </c>
-      <c r="L77" s="2" t="n">
+      <c r="L77" s="1" t="n">
         <v>46080.41190277778</v>
       </c>
       <c r="M77" t="inlineStr">
@@ -8505,7 +8493,7 @@
       <c r="AA77" t="inlineStr"/>
       <c r="AB77" t="inlineStr"/>
       <c r="AC77" t="inlineStr"/>
-      <c r="AD77" s="2" t="n">
+      <c r="AD77" s="1" t="n">
         <v>46080.41190277778</v>
       </c>
       <c r="AE77" t="inlineStr"/>
@@ -8583,7 +8571,7 @@
           <t>Requerimientos</t>
         </is>
       </c>
-      <c r="L78" s="2" t="n">
+      <c r="L78" s="1" t="n">
         <v>46080.41223792824</v>
       </c>
       <c r="M78" t="inlineStr">
@@ -8615,7 +8603,7 @@
       <c r="AA78" t="inlineStr"/>
       <c r="AB78" t="inlineStr"/>
       <c r="AC78" t="inlineStr"/>
-      <c r="AD78" s="2" t="n">
+      <c r="AD78" s="1" t="n">
         <v>46080.41223792824</v>
       </c>
       <c r="AE78" t="inlineStr"/>
@@ -8698,7 +8686,7 @@
           <t>Enviado para Revisión</t>
         </is>
       </c>
-      <c r="S79" s="2" t="n">
+      <c r="S79" s="1" t="n">
         <v>46028.64390934028</v>
       </c>
       <c r="T79" t="inlineStr">
@@ -8717,7 +8705,7 @@
       <c r="AA79" t="inlineStr"/>
       <c r="AB79" t="inlineStr"/>
       <c r="AC79" t="inlineStr"/>
-      <c r="AD79" s="2" t="n">
+      <c r="AD79" s="1" t="n">
         <v>46028.64390934028</v>
       </c>
       <c r="AE79" t="inlineStr"/>
@@ -8791,7 +8779,7 @@
           <t>Requerimientos</t>
         </is>
       </c>
-      <c r="L80" s="2" t="n">
+      <c r="L80" s="1" t="n">
         <v>46071.92375347222</v>
       </c>
       <c r="M80" t="inlineStr">
@@ -8823,7 +8811,7 @@
       <c r="AA80" t="inlineStr"/>
       <c r="AB80" t="inlineStr"/>
       <c r="AC80" t="inlineStr"/>
-      <c r="AD80" s="2" t="n">
+      <c r="AD80" s="1" t="n">
         <v>46071.92375347222</v>
       </c>
       <c r="AE80" t="inlineStr"/>
@@ -8901,7 +8889,7 @@
           <t>Requerimientos</t>
         </is>
       </c>
-      <c r="L81" s="2" t="n">
+      <c r="L81" s="1" t="n">
         <v>46071.9018147801</v>
       </c>
       <c r="M81" t="inlineStr">
@@ -8933,7 +8921,7 @@
       <c r="AA81" t="inlineStr"/>
       <c r="AB81" t="inlineStr"/>
       <c r="AC81" t="inlineStr"/>
-      <c r="AD81" s="2" t="n">
+      <c r="AD81" s="1" t="n">
         <v>46071.9018147801</v>
       </c>
       <c r="AE81" t="inlineStr"/>
@@ -9011,7 +8999,7 @@
           <t>Por el cual ordena el Archivo de un expediente</t>
         </is>
       </c>
-      <c r="L82" s="2" t="n">
+      <c r="L82" s="1" t="n">
         <v>46052.72872369213</v>
       </c>
       <c r="M82" t="inlineStr">
@@ -9043,7 +9031,7 @@
       <c r="AA82" t="inlineStr"/>
       <c r="AB82" t="inlineStr"/>
       <c r="AC82" t="inlineStr"/>
-      <c r="AD82" s="2" t="n">
+      <c r="AD82" s="1" t="n">
         <v>46052.72872369213</v>
       </c>
       <c r="AE82" t="inlineStr"/>
@@ -9121,7 +9109,7 @@
           <t>Por el cual ordena el Archivo de un expediente</t>
         </is>
       </c>
-      <c r="L83" s="2" t="n">
+      <c r="L83" s="1" t="n">
         <v>46064.41688217592</v>
       </c>
       <c r="M83" t="inlineStr"/>
@@ -9145,7 +9133,7 @@
       <c r="AA83" t="inlineStr"/>
       <c r="AB83" t="inlineStr"/>
       <c r="AC83" t="inlineStr"/>
-      <c r="AD83" s="2" t="n">
+      <c r="AD83" s="1" t="n">
         <v>46064.41688217592</v>
       </c>
       <c r="AE83" t="inlineStr"/>
@@ -9219,7 +9207,7 @@
           <t>Requerimientos</t>
         </is>
       </c>
-      <c r="L84" s="2" t="n">
+      <c r="L84" s="1" t="n">
         <v>46065.31646130787</v>
       </c>
       <c r="M84" t="inlineStr">
@@ -9251,7 +9239,7 @@
       <c r="AA84" t="inlineStr"/>
       <c r="AB84" t="inlineStr"/>
       <c r="AC84" t="inlineStr"/>
-      <c r="AD84" s="2" t="n">
+      <c r="AD84" s="1" t="n">
         <v>46065.31646130787</v>
       </c>
       <c r="AE84" t="inlineStr"/>
@@ -9329,7 +9317,7 @@
           <t>Declara el Cumplimiento de Unas Obligaciones</t>
         </is>
       </c>
-      <c r="L85" s="2" t="n">
+      <c r="L85" s="1" t="n">
         <v>46030.72973596065</v>
       </c>
       <c r="M85" t="inlineStr">
@@ -9361,7 +9349,7 @@
       <c r="AA85" t="inlineStr"/>
       <c r="AB85" t="inlineStr"/>
       <c r="AC85" t="inlineStr"/>
-      <c r="AD85" s="2" t="n">
+      <c r="AD85" s="1" t="n">
         <v>46030.72973596065</v>
       </c>
       <c r="AE85" t="inlineStr"/>
@@ -9439,7 +9427,7 @@
           <t>Por el cual ordena el Archivo de un expediente</t>
         </is>
       </c>
-      <c r="L86" s="2" t="n">
+      <c r="L86" s="1" t="n">
         <v>46030.72973052083</v>
       </c>
       <c r="M86" t="inlineStr">
@@ -9471,7 +9459,7 @@
       <c r="AA86" t="inlineStr"/>
       <c r="AB86" t="inlineStr"/>
       <c r="AC86" t="inlineStr"/>
-      <c r="AD86" s="2" t="n">
+      <c r="AD86" s="1" t="n">
         <v>46030.72973052083</v>
       </c>
       <c r="AE86" t="inlineStr"/>
@@ -9549,7 +9537,7 @@
           <t>Aclara Acto Administrativo</t>
         </is>
       </c>
-      <c r="L87" s="2" t="n">
+      <c r="L87" s="1" t="n">
         <v>46093.90440231482</v>
       </c>
       <c r="M87" t="inlineStr">
@@ -9580,7 +9568,7 @@
           <t>Enviado para Revisión</t>
         </is>
       </c>
-      <c r="S87" s="2" t="n">
+      <c r="S87" s="1" t="n">
         <v>46100.39411284722</v>
       </c>
       <c r="T87" t="inlineStr">
@@ -9599,7 +9587,7 @@
       <c r="AA87" t="inlineStr"/>
       <c r="AB87" t="inlineStr"/>
       <c r="AC87" t="inlineStr"/>
-      <c r="AD87" s="2" t="n">
+      <c r="AD87" s="1" t="n">
         <v>46100.39411284722</v>
       </c>
       <c r="AE87" t="inlineStr"/>
@@ -9677,7 +9665,7 @@
           <t>Exoneración de cobro de evaluación y/o seguimiento</t>
         </is>
       </c>
-      <c r="L88" s="2" t="n">
+      <c r="L88" s="1" t="n">
         <v>46099.90026142361</v>
       </c>
       <c r="M88" t="inlineStr">
@@ -9708,7 +9696,7 @@
           <t>Enviado para Revisión</t>
         </is>
       </c>
-      <c r="S88" s="2" t="n">
+      <c r="S88" s="1" t="n">
         <v>46100.4093045949</v>
       </c>
       <c r="T88" t="inlineStr">
@@ -9727,7 +9715,7 @@
       <c r="AA88" t="inlineStr"/>
       <c r="AB88" t="inlineStr"/>
       <c r="AC88" t="inlineStr"/>
-      <c r="AD88" s="2" t="n">
+      <c r="AD88" s="1" t="n">
         <v>46100.4093045949</v>
       </c>
       <c r="AE88" t="inlineStr"/>
@@ -9805,7 +9793,7 @@
           <t>Aclara Acto Administrativo</t>
         </is>
       </c>
-      <c r="L89" s="2" t="n">
+      <c r="L89" s="1" t="n">
         <v>46077.60072172454</v>
       </c>
       <c r="M89" t="inlineStr"/>
@@ -9828,7 +9816,7 @@
           <t>Enviado para Revisión</t>
         </is>
       </c>
-      <c r="S89" s="2" t="n">
+      <c r="S89" s="1" t="n">
         <v>46100.43680690973</v>
       </c>
       <c r="T89" t="inlineStr">
@@ -9847,7 +9835,7 @@
       <c r="AA89" t="inlineStr"/>
       <c r="AB89" t="inlineStr"/>
       <c r="AC89" t="inlineStr"/>
-      <c r="AD89" s="2" t="n">
+      <c r="AD89" s="1" t="n">
         <v>46100.43680690973</v>
       </c>
       <c r="AE89" t="inlineStr"/>
@@ -9921,7 +9909,7 @@
           <t>Aclara Acto Administrativo</t>
         </is>
       </c>
-      <c r="L90" s="2" t="n">
+      <c r="L90" s="1" t="n">
         <v>46083.4502625</v>
       </c>
       <c r="M90" t="inlineStr"/>
@@ -9945,7 +9933,7 @@
       <c r="AA90" t="inlineStr"/>
       <c r="AB90" t="inlineStr"/>
       <c r="AC90" t="inlineStr"/>
-      <c r="AD90" s="2" t="n">
+      <c r="AD90" s="1" t="n">
         <v>46083.4502625</v>
       </c>
       <c r="AE90" t="inlineStr"/>
@@ -10019,7 +10007,7 @@
           <t>Aclara Acto Administrativo</t>
         </is>
       </c>
-      <c r="L91" s="2" t="n">
+      <c r="L91" s="1" t="n">
         <v>46083.45427870371</v>
       </c>
       <c r="M91" t="inlineStr"/>
@@ -10043,7 +10031,7 @@
       <c r="AA91" t="inlineStr"/>
       <c r="AB91" t="inlineStr"/>
       <c r="AC91" t="inlineStr"/>
-      <c r="AD91" s="2" t="n">
+      <c r="AD91" s="1" t="n">
         <v>46083.45427870371</v>
       </c>
       <c r="AE91" t="inlineStr"/>
@@ -10117,7 +10105,7 @@
           <t>Requerimientos</t>
         </is>
       </c>
-      <c r="L92" s="2" t="n">
+      <c r="L92" s="1" t="n">
         <v>46098.91110424769</v>
       </c>
       <c r="M92" t="inlineStr"/>
@@ -10141,7 +10129,7 @@
       <c r="AA92" t="inlineStr"/>
       <c r="AB92" t="inlineStr"/>
       <c r="AC92" t="inlineStr"/>
-      <c r="AD92" s="2" t="n">
+      <c r="AD92" s="1" t="n">
         <v>46098.91110424769</v>
       </c>
       <c r="AE92" t="inlineStr"/>
@@ -10215,7 +10203,7 @@
           <t>Requerimientos</t>
         </is>
       </c>
-      <c r="L93" s="2" t="n">
+      <c r="L93" s="1" t="n">
         <v>46101.89296087963</v>
       </c>
       <c r="M93" t="inlineStr"/>
@@ -10239,7 +10227,7 @@
       <c r="AA93" t="inlineStr"/>
       <c r="AB93" t="inlineStr"/>
       <c r="AC93" t="inlineStr"/>
-      <c r="AD93" s="2" t="n">
+      <c r="AD93" s="1" t="n">
         <v>46101.89296087963</v>
       </c>
       <c r="AE93" t="inlineStr"/>
@@ -10313,7 +10301,7 @@
           <t>Requerimientos</t>
         </is>
       </c>
-      <c r="L94" s="2" t="n">
+      <c r="L94" s="1" t="n">
         <v>46100.39882461805</v>
       </c>
       <c r="M94" t="inlineStr"/>
@@ -10337,7 +10325,7 @@
       <c r="AA94" t="inlineStr"/>
       <c r="AB94" t="inlineStr"/>
       <c r="AC94" t="inlineStr"/>
-      <c r="AD94" s="2" t="n">
+      <c r="AD94" s="1" t="n">
         <v>46100.39882461805</v>
       </c>
       <c r="AE94" t="inlineStr"/>
@@ -10411,7 +10399,7 @@
           <t>Requerimiento y realiza cobro por seguimiento ambiental</t>
         </is>
       </c>
-      <c r="L95" s="2" t="n">
+      <c r="L95" s="1" t="n">
         <v>46091.90538761574</v>
       </c>
       <c r="M95" t="inlineStr"/>
@@ -10435,7 +10423,7 @@
       <c r="AA95" t="inlineStr"/>
       <c r="AB95" t="inlineStr"/>
       <c r="AC95" t="inlineStr"/>
-      <c r="AD95" s="2" t="n">
+      <c r="AD95" s="1" t="n">
         <v>46091.90538761574</v>
       </c>
       <c r="AE95" t="inlineStr"/>
@@ -10509,7 +10497,7 @@
           <t>Requerimientos</t>
         </is>
       </c>
-      <c r="L96" s="2" t="n">
+      <c r="L96" s="1" t="n">
         <v>46100.93431079861</v>
       </c>
       <c r="M96" t="inlineStr"/>
@@ -10533,7 +10521,7 @@
       <c r="AA96" t="inlineStr"/>
       <c r="AB96" t="inlineStr"/>
       <c r="AC96" t="inlineStr"/>
-      <c r="AD96" s="2" t="n">
+      <c r="AD96" s="1" t="n">
         <v>46100.93431079861</v>
       </c>
       <c r="AE96" t="inlineStr"/>
@@ -10607,7 +10595,7 @@
           <t>Aprueba un programa de uso eficiente y ahorro de agua</t>
         </is>
       </c>
-      <c r="L97" s="2" t="n">
+      <c r="L97" s="1" t="n">
         <v>46085.98548614583</v>
       </c>
       <c r="M97" t="inlineStr"/>
@@ -10631,7 +10619,7 @@
       <c r="AA97" t="inlineStr"/>
       <c r="AB97" t="inlineStr"/>
       <c r="AC97" t="inlineStr"/>
-      <c r="AD97" s="2" t="n">
+      <c r="AD97" s="1" t="n">
         <v>46085.98548614583</v>
       </c>
       <c r="AE97" t="inlineStr"/>
@@ -10705,7 +10693,7 @@
           <t>Aclara Acto Administrativo</t>
         </is>
       </c>
-      <c r="L98" s="2" t="n">
+      <c r="L98" s="1" t="n">
         <v>46083.41679259259</v>
       </c>
       <c r="M98" t="inlineStr"/>
@@ -10729,7 +10717,7 @@
       <c r="AA98" t="inlineStr"/>
       <c r="AB98" t="inlineStr"/>
       <c r="AC98" t="inlineStr"/>
-      <c r="AD98" s="2" t="n">
+      <c r="AD98" s="1" t="n">
         <v>46083.41679259259</v>
       </c>
       <c r="AE98" t="inlineStr"/>
@@ -10803,7 +10791,7 @@
           <t>Requerimiento y realiza cobro por seguimiento ambiental</t>
         </is>
       </c>
-      <c r="L99" s="2" t="n">
+      <c r="L99" s="1" t="n">
         <v>46091.93342523148</v>
       </c>
       <c r="M99" t="inlineStr"/>
@@ -10827,7 +10815,7 @@
       <c r="AA99" t="inlineStr"/>
       <c r="AB99" t="inlineStr"/>
       <c r="AC99" t="inlineStr"/>
-      <c r="AD99" s="2" t="n">
+      <c r="AD99" s="1" t="n">
         <v>46091.93342523148</v>
       </c>
       <c r="AE99" t="inlineStr"/>
@@ -10901,7 +10889,7 @@
           <t>Requerimientos</t>
         </is>
       </c>
-      <c r="L100" s="2" t="n">
+      <c r="L100" s="1" t="n">
         <v>46100.84129394676</v>
       </c>
       <c r="M100" t="inlineStr">
@@ -10933,7 +10921,7 @@
       <c r="AA100" t="inlineStr"/>
       <c r="AB100" t="inlineStr"/>
       <c r="AC100" t="inlineStr"/>
-      <c r="AD100" s="2" t="n">
+      <c r="AD100" s="1" t="n">
         <v>46100.84129394676</v>
       </c>
       <c r="AE100" t="inlineStr"/>
@@ -11011,7 +10999,7 @@
           <t>Notificación personal medio electrónico</t>
         </is>
       </c>
-      <c r="L101" s="2" t="n">
+      <c r="L101" s="1" t="n">
         <v>46094.41456284723</v>
       </c>
       <c r="M101" t="inlineStr">
@@ -11043,7 +11031,7 @@
       <c r="AA101" t="inlineStr"/>
       <c r="AB101" t="inlineStr"/>
       <c r="AC101" t="inlineStr"/>
-      <c r="AD101" s="2" t="n">
+      <c r="AD101" s="1" t="n">
         <v>46094.41456284723</v>
       </c>
       <c r="AE101" t="inlineStr"/>
@@ -11121,7 +11109,7 @@
           <t>Requerimientos</t>
         </is>
       </c>
-      <c r="L102" s="2" t="n">
+      <c r="L102" s="1" t="n">
         <v>46091.56697542824</v>
       </c>
       <c r="M102" t="inlineStr"/>
@@ -11145,7 +11133,7 @@
       <c r="AA102" t="inlineStr"/>
       <c r="AB102" t="inlineStr"/>
       <c r="AC102" t="inlineStr"/>
-      <c r="AD102" s="2" t="n">
+      <c r="AD102" s="1" t="n">
         <v>46091.56697542824</v>
       </c>
       <c r="AE102" t="inlineStr"/>
@@ -11219,7 +11207,7 @@
           <t>Notificación personal medio electrónico</t>
         </is>
       </c>
-      <c r="L103" s="2" t="n">
+      <c r="L103" s="1" t="n">
         <v>46094.41535717592</v>
       </c>
       <c r="M103" t="inlineStr">
@@ -11251,7 +11239,7 @@
       <c r="AA103" t="inlineStr"/>
       <c r="AB103" t="inlineStr"/>
       <c r="AC103" t="inlineStr"/>
-      <c r="AD103" s="2" t="n">
+      <c r="AD103" s="1" t="n">
         <v>46094.41535717592</v>
       </c>
       <c r="AE103" t="inlineStr"/>
@@ -11329,7 +11317,7 @@
           <t>Aclara Acto Administrativo</t>
         </is>
       </c>
-      <c r="L104" s="2" t="n">
+      <c r="L104" s="1" t="n">
         <v>46083.44661288195</v>
       </c>
       <c r="M104" t="inlineStr"/>
@@ -11353,7 +11341,7 @@
       <c r="AA104" t="inlineStr"/>
       <c r="AB104" t="inlineStr"/>
       <c r="AC104" t="inlineStr"/>
-      <c r="AD104" s="2" t="n">
+      <c r="AD104" s="1" t="n">
         <v>46083.44661288195</v>
       </c>
       <c r="AE104" t="inlineStr"/>
@@ -11427,7 +11415,7 @@
           <t>Aclara Acto Administrativo</t>
         </is>
       </c>
-      <c r="L105" s="2" t="n">
+      <c r="L105" s="1" t="n">
         <v>46083.44158769676</v>
       </c>
       <c r="M105" t="inlineStr"/>
@@ -11451,7 +11439,7 @@
       <c r="AA105" t="inlineStr"/>
       <c r="AB105" t="inlineStr"/>
       <c r="AC105" t="inlineStr"/>
-      <c r="AD105" s="2" t="n">
+      <c r="AD105" s="1" t="n">
         <v>46083.44158769676</v>
       </c>
       <c r="AE105" t="inlineStr"/>
@@ -11525,7 +11513,7 @@
           <t>Oficio de citación</t>
         </is>
       </c>
-      <c r="L106" s="2" t="n">
+      <c r="L106" s="1" t="n">
         <v>46094.4164028588</v>
       </c>
       <c r="M106" t="inlineStr">
@@ -11557,7 +11545,7 @@
       <c r="AA106" t="inlineStr"/>
       <c r="AB106" t="inlineStr"/>
       <c r="AC106" t="inlineStr"/>
-      <c r="AD106" s="2" t="n">
+      <c r="AD106" s="1" t="n">
         <v>46094.4164028588</v>
       </c>
       <c r="AE106" t="inlineStr"/>
@@ -11635,7 +11623,7 @@
           <t>Aclara Acto Administrativo</t>
         </is>
       </c>
-      <c r="L107" s="2" t="n">
+      <c r="L107" s="1" t="n">
         <v>46081.87232696759</v>
       </c>
       <c r="M107" t="inlineStr"/>
@@ -11659,7 +11647,7 @@
       <c r="AA107" t="inlineStr"/>
       <c r="AB107" t="inlineStr"/>
       <c r="AC107" t="inlineStr"/>
-      <c r="AD107" s="2" t="n">
+      <c r="AD107" s="1" t="n">
         <v>46081.87232696759</v>
       </c>
       <c r="AE107" t="inlineStr"/>
@@ -11733,7 +11721,7 @@
           <t>Aclara Acto Administrativo</t>
         </is>
       </c>
-      <c r="L108" s="2" t="n">
+      <c r="L108" s="1" t="n">
         <v>46077.55379672454</v>
       </c>
       <c r="M108" t="inlineStr"/>
@@ -11757,7 +11745,7 @@
       <c r="AA108" t="inlineStr"/>
       <c r="AB108" t="inlineStr"/>
       <c r="AC108" t="inlineStr"/>
-      <c r="AD108" s="2" t="n">
+      <c r="AD108" s="1" t="n">
         <v>46077.55379672454</v>
       </c>
       <c r="AE108" t="inlineStr"/>
@@ -11831,7 +11819,7 @@
           <t>Aclara Acto Administrativo</t>
         </is>
       </c>
-      <c r="L109" s="2" t="n">
+      <c r="L109" s="1" t="n">
         <v>46077.7154929051</v>
       </c>
       <c r="M109" t="inlineStr"/>
@@ -11855,7 +11843,7 @@
       <c r="AA109" t="inlineStr"/>
       <c r="AB109" t="inlineStr"/>
       <c r="AC109" t="inlineStr"/>
-      <c r="AD109" s="2" t="n">
+      <c r="AD109" s="1" t="n">
         <v>46077.7154929051</v>
       </c>
       <c r="AE109" t="inlineStr"/>
@@ -11929,7 +11917,7 @@
           <t>Aclara Acto Administrativo</t>
         </is>
       </c>
-      <c r="L110" s="2" t="n">
+      <c r="L110" s="1" t="n">
         <v>46077.65739398148</v>
       </c>
       <c r="M110" t="inlineStr"/>
@@ -11953,7 +11941,7 @@
       <c r="AA110" t="inlineStr"/>
       <c r="AB110" t="inlineStr"/>
       <c r="AC110" t="inlineStr"/>
-      <c r="AD110" s="2" t="n">
+      <c r="AD110" s="1" t="n">
         <v>46077.65739398148</v>
       </c>
       <c r="AE110" t="inlineStr"/>
@@ -12027,7 +12015,7 @@
           <t>Aclara Acto Administrativo</t>
         </is>
       </c>
-      <c r="L111" s="2" t="n">
+      <c r="L111" s="1" t="n">
         <v>46075.72491793981</v>
       </c>
       <c r="M111" t="inlineStr"/>
@@ -12051,7 +12039,7 @@
       <c r="AA111" t="inlineStr"/>
       <c r="AB111" t="inlineStr"/>
       <c r="AC111" t="inlineStr"/>
-      <c r="AD111" s="2" t="n">
+      <c r="AD111" s="1" t="n">
         <v>46075.72491793981</v>
       </c>
       <c r="AE111" t="inlineStr"/>
@@ -12125,7 +12113,7 @@
           <t>Aclara Acto Administrativo</t>
         </is>
       </c>
-      <c r="L112" s="2" t="n">
+      <c r="L112" s="1" t="n">
         <v>46075.63706512732</v>
       </c>
       <c r="M112" t="inlineStr"/>
@@ -12149,7 +12137,7 @@
       <c r="AA112" t="inlineStr"/>
       <c r="AB112" t="inlineStr"/>
       <c r="AC112" t="inlineStr"/>
-      <c r="AD112" s="2" t="n">
+      <c r="AD112" s="1" t="n">
         <v>46075.63706512732</v>
       </c>
       <c r="AE112" t="inlineStr"/>
@@ -12188,37 +12176,37 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>nombre_persona</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>estado_pelota_caliente</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>total_expedientes</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>total_registros</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>con_sae</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>con_preradicado</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>con_radicado</t>
         </is>
@@ -12268,13 +12256,13 @@
       <c r="D3" t="n">
         <v>1</v>
       </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G3" t="n">
+      <c r="E3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12349,13 +12337,13 @@
       <c r="D6" t="n">
         <v>1</v>
       </c>
-      <c r="E6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" t="n">
+      <c r="E6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G6" t="b">
         <v>1</v>
       </c>
     </row>
@@ -12403,13 +12391,13 @@
       <c r="D8" t="n">
         <v>1</v>
       </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" t="n">
+      <c r="E8" t="b">
+        <v>0</v>
+      </c>
+      <c r="F8" t="b">
+        <v>1</v>
+      </c>
+      <c r="G8" t="b">
         <v>0</v>
       </c>
     </row>
@@ -12430,13 +12418,13 @@
       <c r="D9" t="n">
         <v>1</v>
       </c>
-      <c r="E9" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" t="n">
+      <c r="E9" t="b">
+        <v>1</v>
+      </c>
+      <c r="F9" t="b">
+        <v>0</v>
+      </c>
+      <c r="G9" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>